<commit_message>
2 new auth-login tests are added, readme is updated
</commit_message>
<xml_diff>
--- a/Check_list.xlsx
+++ b/Check_list.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Чеклист" sheetId="1" state="visible" r:id="rId2"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="144">
   <si>
     <t xml:space="preserve">Проект</t>
   </si>
@@ -125,7 +125,7 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">Успешная авторизация, но с большой задержкой ~ 10 сек</t>
+    <t xml:space="preserve">Успешная авторизация, но с большой задержкой ~ 5 сек</t>
   </si>
   <si>
     <t xml:space="preserve">SD-5</t>
@@ -173,6 +173,9 @@
     <t xml:space="preserve">SD-12</t>
   </si>
   <si>
+    <t xml:space="preserve">Повторная попытка авторизации после неудачной первой</t>
+  </si>
+  <si>
     <t xml:space="preserve">SD-13</t>
   </si>
   <si>
@@ -568,6 +571,27 @@
     </r>
   </si>
   <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="204"/>
+      </rPr>
+      <t xml:space="preserve">В поле Username появилась надпись visual</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="204"/>
+      </rPr>
+      <t xml:space="preserve">_user</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">SD-6.2</t>
   </si>
   <si>
@@ -743,6 +767,51 @@
   </si>
   <si>
     <t xml:space="preserve">SD-11.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SD-12.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Выполнить шаги SD-11.1 — SD-11.3</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="204"/>
+      </rPr>
+      <t xml:space="preserve">На форме появляется всплывающее сообщение об ошибке: «Epic sadface: Username and password do not match any user in this service</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="204"/>
+      </rPr>
+      <t xml:space="preserve">». Авторизация не происходит</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">SD-12.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Закрыть всплывающее сообщение нажатием на белый крестик в правом верхнем углу сообщения об ошибке</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Сообщение об ошибке исчезло, поля ввода очистились от введённых ранее значений</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SD-12.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Выполнить шаги SD-1.1 — SD-1.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Успешная авторизация, загружается страница магазина</t>
   </si>
 </sst>
 </file>
@@ -845,7 +914,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="12">
+  <borders count="15">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
@@ -891,6 +960,15 @@
       <top style="thin">
         <color rgb="FF666666"/>
       </top>
+      <bottom style="thin">
+        <color rgb="FF666666"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
       <bottom style="thin">
         <color rgb="FF666666"/>
       </bottom>
@@ -956,6 +1034,20 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right style="thin"/>
+      <top/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="20">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -982,7 +1074,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="36">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1019,19 +1111,19 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1039,7 +1131,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1067,7 +1167,7 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1075,14 +1175,14 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1091,15 +1191,27 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="13" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1432,88 +1544,98 @@
         <v>16</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="1" t="s">
+    <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="C18" s="9"/>
-      <c r="D18" s="9"/>
+      <c r="B18" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C18" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="E18" s="8" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="C19" s="9"/>
-      <c r="D19" s="9"/>
+        <v>42</v>
+      </c>
+      <c r="C19" s="11"/>
+      <c r="D19" s="11"/>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="C20" s="9"/>
-      <c r="D20" s="9"/>
+        <v>43</v>
+      </c>
+      <c r="C20" s="11"/>
+      <c r="D20" s="11"/>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="C21" s="9"/>
-      <c r="D21" s="9"/>
+        <v>44</v>
+      </c>
+      <c r="C21" s="11"/>
+      <c r="D21" s="11"/>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="C22" s="9"/>
-      <c r="D22" s="9"/>
+        <v>45</v>
+      </c>
+      <c r="C22" s="11"/>
+      <c r="D22" s="11"/>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="C23" s="9"/>
-      <c r="D23" s="9"/>
+        <v>46</v>
+      </c>
+      <c r="C23" s="11"/>
+      <c r="D23" s="11"/>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="C24" s="9"/>
-      <c r="D24" s="9"/>
+        <v>47</v>
+      </c>
+      <c r="C24" s="11"/>
+      <c r="D24" s="11"/>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="C25" s="9"/>
-      <c r="D25" s="9"/>
+        <v>48</v>
+      </c>
+      <c r="C25" s="11"/>
+      <c r="D25" s="11"/>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="C26" s="9"/>
-      <c r="D26" s="9"/>
+        <v>49</v>
+      </c>
+      <c r="C26" s="11"/>
+      <c r="D26" s="11"/>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C27" s="9"/>
-      <c r="D27" s="9"/>
+      <c r="C27" s="11"/>
+      <c r="D27" s="11"/>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C28" s="9"/>
-      <c r="D28" s="9"/>
+      <c r="C28" s="11"/>
+      <c r="D28" s="11"/>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C29" s="9"/>
-      <c r="D29" s="9"/>
+      <c r="C29" s="11"/>
+      <c r="D29" s="11"/>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C30" s="9"/>
-      <c r="D30" s="9"/>
+      <c r="C30" s="11"/>
+      <c r="D30" s="11"/>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C31" s="9"/>
-      <c r="D31" s="9"/>
+      <c r="C31" s="11"/>
+      <c r="D31" s="11"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -1539,54 +1661,54 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="10" t="s">
-        <v>50</v>
-      </c>
-      <c r="B3" s="10" t="s">
+      <c r="A3" s="12" t="s">
         <v>51</v>
       </c>
+      <c r="B3" s="12" t="s">
+        <v>52</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="B4" s="12" t="s">
+      <c r="A4" s="13" t="s">
         <v>53</v>
       </c>
+      <c r="B4" s="14" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="11" t="s">
-        <v>54</v>
-      </c>
-      <c r="B5" s="12"/>
+      <c r="A5" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="B5" s="14"/>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="11" t="s">
-        <v>55</v>
-      </c>
-      <c r="B6" s="12"/>
+      <c r="A6" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="B6" s="14"/>
     </row>
     <row r="7" customFormat="false" ht="23.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="11" t="s">
-        <v>56</v>
-      </c>
-      <c r="B7" s="12"/>
+      <c r="A7" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="B7" s="14"/>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="11" t="s">
-        <v>57</v>
-      </c>
-      <c r="B8" s="12"/>
+      <c r="A8" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="B8" s="14"/>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="13" t="s">
-        <v>58</v>
-      </c>
-      <c r="B9" s="14"/>
+      <c r="A9" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="B9" s="16"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -1623,7 +1745,7 @@
       <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="15"/>
+      <c r="C1" s="17"/>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
@@ -1632,14 +1754,14 @@
       <c r="B2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="15"/>
+      <c r="C2" s="17"/>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B3" s="2"/>
-      <c r="C3" s="15"/>
+      <c r="C3" s="17"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3"/>
@@ -1647,13 +1769,13 @@
       <c r="C4" s="3"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="16" t="s">
-        <v>59</v>
-      </c>
-      <c r="B5" s="16" t="s">
+      <c r="A5" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="B5" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="17"/>
+      <c r="C5" s="19"/>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3"/>
@@ -1662,731 +1784,755 @@
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F7" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="G7" s="18"/>
+      <c r="G7" s="20"/>
     </row>
     <row r="8" customFormat="false" ht="34.55" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="19" t="s">
+      <c r="A8" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="20" t="s">
+      <c r="B8" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="C8" s="20" t="s">
-        <v>65</v>
-      </c>
-      <c r="D8" s="20" t="s">
+      <c r="C8" s="22" t="s">
         <v>66</v>
       </c>
-      <c r="E8" s="19" t="s">
+      <c r="D8" s="22" t="s">
         <v>67</v>
       </c>
-      <c r="F8" s="21" t="s">
+      <c r="E8" s="21" t="s">
         <v>68</v>
       </c>
-      <c r="G8" s="19"/>
+      <c r="F8" s="23" t="s">
+        <v>69</v>
+      </c>
+      <c r="G8" s="21"/>
     </row>
     <row r="9" customFormat="false" ht="24.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="22"/>
-      <c r="B9" s="22"/>
-      <c r="C9" s="22"/>
-      <c r="D9" s="20" t="s">
+      <c r="A9" s="24"/>
+      <c r="B9" s="24"/>
+      <c r="C9" s="24"/>
+      <c r="D9" s="22" t="s">
+        <v>70</v>
+      </c>
+      <c r="E9" s="21" t="s">
+        <v>71</v>
+      </c>
+      <c r="F9" s="23" t="s">
+        <v>72</v>
+      </c>
+      <c r="G9" s="24"/>
+    </row>
+    <row r="10" customFormat="false" ht="29.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="24"/>
+      <c r="B10" s="24"/>
+      <c r="C10" s="24"/>
+      <c r="D10" s="22" t="s">
+        <v>73</v>
+      </c>
+      <c r="E10" s="24" t="s">
+        <v>74</v>
+      </c>
+      <c r="F10" s="23" t="s">
+        <v>75</v>
+      </c>
+      <c r="G10" s="24"/>
+    </row>
+    <row r="11" customFormat="false" ht="24.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="25" t="s">
+        <v>17</v>
+      </c>
+      <c r="B11" s="25" t="s">
+        <v>18</v>
+      </c>
+      <c r="C11" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="D11" s="25" t="s">
+        <v>76</v>
+      </c>
+      <c r="E11" s="25" t="s">
+        <v>77</v>
+      </c>
+      <c r="F11" s="26" t="s">
+        <v>78</v>
+      </c>
+      <c r="G11" s="27"/>
+    </row>
+    <row r="12" customFormat="false" ht="24.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="24"/>
+      <c r="B12" s="24"/>
+      <c r="C12" s="24"/>
+      <c r="D12" s="28" t="s">
+        <v>79</v>
+      </c>
+      <c r="E12" s="21" t="s">
+        <v>71</v>
+      </c>
+      <c r="F12" s="23" t="s">
+        <v>72</v>
+      </c>
+      <c r="G12" s="24"/>
+    </row>
+    <row r="13" customFormat="false" ht="65.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="24"/>
+      <c r="B13" s="24"/>
+      <c r="C13" s="24"/>
+      <c r="D13" s="28" t="s">
+        <v>80</v>
+      </c>
+      <c r="E13" s="24" t="s">
+        <v>74</v>
+      </c>
+      <c r="F13" s="23" t="s">
+        <v>81</v>
+      </c>
+      <c r="G13" s="24"/>
+    </row>
+    <row r="14" customFormat="false" ht="51.55" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="29" t="s">
+        <v>20</v>
+      </c>
+      <c r="B14" s="29" t="s">
+        <v>21</v>
+      </c>
+      <c r="C14" s="29" t="s">
+        <v>66</v>
+      </c>
+      <c r="D14" s="29" t="s">
+        <v>82</v>
+      </c>
+      <c r="E14" s="29" t="s">
+        <v>83</v>
+      </c>
+      <c r="F14" s="30" t="s">
+        <v>84</v>
+      </c>
+      <c r="G14" s="28"/>
+    </row>
+    <row r="15" customFormat="false" ht="24.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="24"/>
+      <c r="B15" s="24"/>
+      <c r="C15" s="24"/>
+      <c r="D15" s="24" t="s">
+        <v>85</v>
+      </c>
+      <c r="E15" s="21" t="s">
+        <v>71</v>
+      </c>
+      <c r="F15" s="23" t="s">
+        <v>86</v>
+      </c>
+      <c r="G15" s="24"/>
+    </row>
+    <row r="16" customFormat="false" ht="35.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="24"/>
+      <c r="B16" s="24"/>
+      <c r="C16" s="24"/>
+      <c r="D16" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="E16" s="21" t="s">
+        <v>74</v>
+      </c>
+      <c r="F16" s="23" t="s">
+        <v>88</v>
+      </c>
+      <c r="G16" s="24"/>
+    </row>
+    <row r="17" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="29" t="s">
+        <v>23</v>
+      </c>
+      <c r="B17" s="31" t="s">
+        <v>89</v>
+      </c>
+      <c r="C17" s="29" t="s">
+        <v>66</v>
+      </c>
+      <c r="D17" s="29" t="s">
+        <v>90</v>
+      </c>
+      <c r="E17" s="29" t="s">
+        <v>91</v>
+      </c>
+      <c r="F17" s="30" t="s">
+        <v>92</v>
+      </c>
+      <c r="G17" s="28"/>
+    </row>
+    <row r="18" customFormat="false" ht="24.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="24"/>
+      <c r="B18" s="24"/>
+      <c r="C18" s="24"/>
+      <c r="D18" s="24" t="s">
+        <v>93</v>
+      </c>
+      <c r="E18" s="21" t="s">
+        <v>71</v>
+      </c>
+      <c r="F18" s="23" t="s">
+        <v>86</v>
+      </c>
+      <c r="G18" s="24"/>
+    </row>
+    <row r="19" customFormat="false" ht="24.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="24"/>
+      <c r="B19" s="24"/>
+      <c r="C19" s="24"/>
+      <c r="D19" s="24" t="s">
+        <v>94</v>
+      </c>
+      <c r="E19" s="21" t="s">
+        <v>74</v>
+      </c>
+      <c r="F19" s="23" t="s">
+        <v>95</v>
+      </c>
+      <c r="G19" s="24"/>
+    </row>
+    <row r="20" customFormat="false" ht="24.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="29" t="s">
+        <v>26</v>
+      </c>
+      <c r="B20" s="31" t="s">
+        <v>96</v>
+      </c>
+      <c r="C20" s="29" t="s">
+        <v>66</v>
+      </c>
+      <c r="D20" s="29" t="s">
+        <v>97</v>
+      </c>
+      <c r="E20" s="29" t="s">
+        <v>98</v>
+      </c>
+      <c r="F20" s="30" t="s">
+        <v>99</v>
+      </c>
+      <c r="G20" s="28"/>
+    </row>
+    <row r="21" customFormat="false" ht="24.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="24"/>
+      <c r="B21" s="24"/>
+      <c r="C21" s="24"/>
+      <c r="D21" s="24" t="s">
+        <v>100</v>
+      </c>
+      <c r="E21" s="21" t="s">
+        <v>71</v>
+      </c>
+      <c r="F21" s="23" t="s">
+        <v>86</v>
+      </c>
+      <c r="G21" s="24"/>
+    </row>
+    <row r="22" customFormat="false" ht="24.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="24"/>
+      <c r="B22" s="24"/>
+      <c r="C22" s="24"/>
+      <c r="D22" s="24" t="s">
+        <v>101</v>
+      </c>
+      <c r="E22" s="21" t="s">
+        <v>74</v>
+      </c>
+      <c r="F22" s="23" t="s">
+        <v>75</v>
+      </c>
+      <c r="G22" s="24"/>
+    </row>
+    <row r="23" customFormat="false" ht="24.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="B23" s="31" t="s">
+        <v>102</v>
+      </c>
+      <c r="C23" s="29" t="s">
+        <v>66</v>
+      </c>
+      <c r="D23" s="29" t="s">
+        <v>103</v>
+      </c>
+      <c r="E23" s="29" t="s">
+        <v>104</v>
+      </c>
+      <c r="F23" s="30" t="s">
+        <v>105</v>
+      </c>
+      <c r="G23" s="28"/>
+    </row>
+    <row r="24" customFormat="false" ht="24.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="24"/>
+      <c r="B24" s="24"/>
+      <c r="C24" s="24"/>
+      <c r="D24" s="24" t="s">
+        <v>106</v>
+      </c>
+      <c r="E24" s="21" t="s">
+        <v>71</v>
+      </c>
+      <c r="F24" s="23" t="s">
+        <v>86</v>
+      </c>
+      <c r="G24" s="24"/>
+    </row>
+    <row r="25" customFormat="false" ht="24.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="24"/>
+      <c r="B25" s="24"/>
+      <c r="C25" s="24"/>
+      <c r="D25" s="24" t="s">
+        <v>107</v>
+      </c>
+      <c r="E25" s="21" t="s">
+        <v>74</v>
+      </c>
+      <c r="F25" s="23" t="s">
+        <v>75</v>
+      </c>
+      <c r="G25" s="24"/>
+    </row>
+    <row r="26" customFormat="false" ht="24.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="29" t="s">
+        <v>30</v>
+      </c>
+      <c r="B26" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="C26" s="29" t="s">
+        <v>66</v>
+      </c>
+      <c r="D26" s="29" t="s">
+        <v>108</v>
+      </c>
+      <c r="E26" s="29" t="s">
+        <v>109</v>
+      </c>
+      <c r="F26" s="30" t="s">
+        <v>110</v>
+      </c>
+      <c r="G26" s="24"/>
+    </row>
+    <row r="27" customFormat="false" ht="24.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="24"/>
+      <c r="B27" s="24"/>
+      <c r="C27" s="24"/>
+      <c r="D27" s="24" t="s">
+        <v>111</v>
+      </c>
+      <c r="E27" s="21" t="s">
+        <v>71</v>
+      </c>
+      <c r="F27" s="23" t="s">
+        <v>86</v>
+      </c>
+      <c r="G27" s="24"/>
+    </row>
+    <row r="28" customFormat="false" ht="47.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="24"/>
+      <c r="B28" s="24"/>
+      <c r="C28" s="24"/>
+      <c r="D28" s="24" t="s">
+        <v>112</v>
+      </c>
+      <c r="E28" s="21" t="s">
+        <v>74</v>
+      </c>
+      <c r="F28" s="23" t="s">
+        <v>113</v>
+      </c>
+      <c r="G28" s="24"/>
+    </row>
+    <row r="29" customFormat="false" ht="24.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="29" t="s">
+        <v>32</v>
+      </c>
+      <c r="B29" s="29" t="s">
+        <v>33</v>
+      </c>
+      <c r="C29" s="29" t="s">
+        <v>66</v>
+      </c>
+      <c r="D29" s="29" t="s">
+        <v>114</v>
+      </c>
+      <c r="E29" s="29" t="s">
+        <v>115</v>
+      </c>
+      <c r="F29" s="30" t="s">
         <v>69</v>
       </c>
-      <c r="E9" s="19" t="s">
-        <v>70</v>
-      </c>
-      <c r="F9" s="21" t="s">
+      <c r="G29" s="24"/>
+    </row>
+    <row r="30" customFormat="false" ht="12.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="24"/>
+      <c r="B30" s="24"/>
+      <c r="C30" s="24"/>
+      <c r="D30" s="24" t="s">
+        <v>116</v>
+      </c>
+      <c r="E30" s="21" t="s">
+        <v>117</v>
+      </c>
+      <c r="F30" s="23" t="s">
+        <v>118</v>
+      </c>
+      <c r="G30" s="24"/>
+    </row>
+    <row r="31" customFormat="false" ht="47.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="24"/>
+      <c r="B31" s="24"/>
+      <c r="C31" s="24"/>
+      <c r="D31" s="24" t="s">
+        <v>119</v>
+      </c>
+      <c r="E31" s="21" t="s">
+        <v>74</v>
+      </c>
+      <c r="F31" s="23" t="s">
+        <v>120</v>
+      </c>
+      <c r="G31" s="24"/>
+    </row>
+    <row r="32" customFormat="false" ht="87.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="29" t="s">
+        <v>34</v>
+      </c>
+      <c r="B32" s="29" t="s">
+        <v>35</v>
+      </c>
+      <c r="C32" s="29" t="s">
+        <v>66</v>
+      </c>
+      <c r="D32" s="29" t="s">
+        <v>121</v>
+      </c>
+      <c r="E32" s="29" t="s">
+        <v>122</v>
+      </c>
+      <c r="F32" s="30" t="s">
+        <v>123</v>
+      </c>
+      <c r="G32" s="24"/>
+    </row>
+    <row r="33" customFormat="false" ht="24.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="24"/>
+      <c r="B33" s="24"/>
+      <c r="C33" s="24"/>
+      <c r="D33" s="24" t="s">
+        <v>124</v>
+      </c>
+      <c r="E33" s="21" t="s">
         <v>71</v>
       </c>
-      <c r="G9" s="22"/>
-    </row>
-    <row r="10" customFormat="false" ht="29.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="22"/>
-      <c r="B10" s="22"/>
-      <c r="C10" s="22"/>
-      <c r="D10" s="20" t="s">
-        <v>72</v>
-      </c>
-      <c r="E10" s="22" t="s">
-        <v>73</v>
-      </c>
-      <c r="F10" s="21" t="s">
+      <c r="F33" s="23" t="s">
+        <v>86</v>
+      </c>
+      <c r="G33" s="24"/>
+    </row>
+    <row r="34" customFormat="false" ht="59" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="24"/>
+      <c r="B34" s="24"/>
+      <c r="C34" s="24"/>
+      <c r="D34" s="24" t="s">
+        <v>125</v>
+      </c>
+      <c r="E34" s="21" t="s">
         <v>74</v>
       </c>
-      <c r="G10" s="22"/>
-    </row>
-    <row r="11" customFormat="false" ht="24.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="23" t="s">
-        <v>17</v>
-      </c>
-      <c r="B11" s="23" t="s">
-        <v>18</v>
-      </c>
-      <c r="C11" s="23" t="s">
-        <v>65</v>
-      </c>
-      <c r="D11" s="23" t="s">
-        <v>75</v>
-      </c>
-      <c r="E11" s="23" t="s">
-        <v>76</v>
-      </c>
-      <c r="F11" s="24" t="s">
-        <v>77</v>
-      </c>
-      <c r="G11" s="25"/>
-    </row>
-    <row r="12" customFormat="false" ht="24.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="22"/>
-      <c r="B12" s="22"/>
-      <c r="C12" s="22"/>
-      <c r="D12" s="26" t="s">
-        <v>78</v>
-      </c>
-      <c r="E12" s="19" t="s">
-        <v>70</v>
-      </c>
-      <c r="F12" s="21" t="s">
-        <v>71</v>
-      </c>
-      <c r="G12" s="22"/>
-    </row>
-    <row r="13" customFormat="false" ht="65.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="22"/>
-      <c r="B13" s="22"/>
-      <c r="C13" s="22"/>
-      <c r="D13" s="26" t="s">
-        <v>79</v>
-      </c>
-      <c r="E13" s="22" t="s">
-        <v>73</v>
-      </c>
-      <c r="F13" s="21" t="s">
-        <v>80</v>
-      </c>
-      <c r="G13" s="22"/>
-    </row>
-    <row r="14" customFormat="false" ht="51.55" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="27" t="s">
-        <v>20</v>
-      </c>
-      <c r="B14" s="27" t="s">
-        <v>21</v>
-      </c>
-      <c r="C14" s="27" t="s">
-        <v>65</v>
-      </c>
-      <c r="D14" s="27" t="s">
-        <v>81</v>
-      </c>
-      <c r="E14" s="27" t="s">
-        <v>82</v>
-      </c>
-      <c r="F14" s="28" t="s">
-        <v>83</v>
-      </c>
-      <c r="G14" s="26"/>
-    </row>
-    <row r="15" customFormat="false" ht="24.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="22"/>
-      <c r="B15" s="22"/>
-      <c r="C15" s="22"/>
-      <c r="D15" s="22" t="s">
-        <v>84</v>
-      </c>
-      <c r="E15" s="19" t="s">
-        <v>70</v>
-      </c>
-      <c r="F15" s="21" t="s">
-        <v>85</v>
-      </c>
-      <c r="G15" s="22"/>
-    </row>
-    <row r="16" customFormat="false" ht="35.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="22"/>
-      <c r="B16" s="22"/>
-      <c r="C16" s="22"/>
-      <c r="D16" s="22" t="s">
+      <c r="F34" s="23" t="s">
+        <v>126</v>
+      </c>
+      <c r="G34" s="24"/>
+    </row>
+    <row r="35" customFormat="false" ht="35.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="29" t="s">
+        <v>36</v>
+      </c>
+      <c r="B35" s="29" t="s">
+        <v>37</v>
+      </c>
+      <c r="C35" s="29" t="s">
+        <v>66</v>
+      </c>
+      <c r="D35" s="29" t="s">
+        <v>127</v>
+      </c>
+      <c r="E35" s="29" t="s">
+        <v>115</v>
+      </c>
+      <c r="F35" s="30" t="s">
+        <v>128</v>
+      </c>
+      <c r="G35" s="24"/>
+    </row>
+    <row r="36" customFormat="false" ht="71.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="24"/>
+      <c r="B36" s="24"/>
+      <c r="C36" s="24"/>
+      <c r="D36" s="24" t="s">
+        <v>129</v>
+      </c>
+      <c r="E36" s="21" t="s">
+        <v>130</v>
+      </c>
+      <c r="F36" s="23" t="s">
         <v>86</v>
       </c>
-      <c r="E16" s="19" t="s">
-        <v>73</v>
-      </c>
-      <c r="F16" s="21" t="s">
-        <v>87</v>
-      </c>
-      <c r="G16" s="22"/>
-    </row>
-    <row r="17" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="27" t="s">
-        <v>23</v>
-      </c>
-      <c r="B17" s="29" t="s">
-        <v>88</v>
-      </c>
-      <c r="C17" s="27" t="s">
-        <v>65</v>
-      </c>
-      <c r="D17" s="27" t="s">
-        <v>89</v>
-      </c>
-      <c r="E17" s="27" t="s">
-        <v>90</v>
-      </c>
-      <c r="F17" s="28" t="s">
-        <v>91</v>
-      </c>
-      <c r="G17" s="26"/>
-    </row>
-    <row r="18" customFormat="false" ht="24.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="22"/>
-      <c r="B18" s="22"/>
-      <c r="C18" s="22"/>
-      <c r="D18" s="22" t="s">
-        <v>92</v>
-      </c>
-      <c r="E18" s="19" t="s">
-        <v>70</v>
-      </c>
-      <c r="F18" s="21" t="s">
-        <v>85</v>
-      </c>
-      <c r="G18" s="22"/>
-    </row>
-    <row r="19" customFormat="false" ht="24.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="22"/>
-      <c r="B19" s="22"/>
-      <c r="C19" s="22"/>
-      <c r="D19" s="22" t="s">
-        <v>93</v>
-      </c>
-      <c r="E19" s="19" t="s">
-        <v>73</v>
-      </c>
-      <c r="F19" s="21" t="s">
-        <v>94</v>
-      </c>
-      <c r="G19" s="22"/>
-    </row>
-    <row r="20" customFormat="false" ht="24.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="27" t="s">
-        <v>26</v>
-      </c>
-      <c r="B20" s="29" t="s">
-        <v>95</v>
-      </c>
-      <c r="C20" s="27" t="s">
-        <v>65</v>
-      </c>
-      <c r="D20" s="27" t="s">
-        <v>96</v>
-      </c>
-      <c r="E20" s="27" t="s">
-        <v>97</v>
-      </c>
-      <c r="F20" s="28" t="s">
-        <v>98</v>
-      </c>
-      <c r="G20" s="26"/>
-    </row>
-    <row r="21" customFormat="false" ht="24.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="22"/>
-      <c r="B21" s="22"/>
-      <c r="C21" s="22"/>
-      <c r="D21" s="22" t="s">
-        <v>99</v>
-      </c>
-      <c r="E21" s="19" t="s">
-        <v>70</v>
-      </c>
-      <c r="F21" s="21" t="s">
-        <v>85</v>
-      </c>
-      <c r="G21" s="22"/>
-    </row>
-    <row r="22" customFormat="false" ht="24.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="22"/>
-      <c r="B22" s="22"/>
-      <c r="C22" s="22"/>
-      <c r="D22" s="22" t="s">
-        <v>100</v>
-      </c>
-      <c r="E22" s="19" t="s">
-        <v>73</v>
-      </c>
-      <c r="F22" s="21" t="s">
+      <c r="G36" s="24"/>
+    </row>
+    <row r="37" customFormat="false" ht="59" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="24"/>
+      <c r="B37" s="24"/>
+      <c r="C37" s="24"/>
+      <c r="D37" s="24" t="s">
+        <v>131</v>
+      </c>
+      <c r="E37" s="21" t="s">
         <v>74</v>
       </c>
-      <c r="G22" s="22"/>
-    </row>
-    <row r="23" customFormat="false" ht="24.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="27" t="s">
-        <v>28</v>
-      </c>
-      <c r="B23" s="29" t="s">
-        <v>101</v>
-      </c>
-      <c r="C23" s="27" t="s">
-        <v>65</v>
-      </c>
-      <c r="D23" s="27" t="s">
-        <v>102</v>
-      </c>
-      <c r="E23" s="27" t="s">
-        <v>103</v>
-      </c>
-      <c r="F23" s="28" t="s">
-        <v>98</v>
-      </c>
-      <c r="G23" s="26"/>
-    </row>
-    <row r="24" customFormat="false" ht="24.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="22"/>
-      <c r="B24" s="22"/>
-      <c r="C24" s="22"/>
-      <c r="D24" s="22" t="s">
-        <v>104</v>
-      </c>
-      <c r="E24" s="19" t="s">
-        <v>70</v>
-      </c>
-      <c r="F24" s="21" t="s">
-        <v>85</v>
-      </c>
-      <c r="G24" s="22"/>
-    </row>
-    <row r="25" customFormat="false" ht="24.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="22"/>
-      <c r="B25" s="22"/>
-      <c r="C25" s="22"/>
-      <c r="D25" s="22" t="s">
-        <v>105</v>
-      </c>
-      <c r="E25" s="19" t="s">
-        <v>73</v>
-      </c>
-      <c r="F25" s="21" t="s">
+      <c r="F37" s="23" t="s">
+        <v>126</v>
+      </c>
+      <c r="G37" s="24"/>
+    </row>
+    <row r="38" customFormat="false" ht="87.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="29" t="s">
+        <v>38</v>
+      </c>
+      <c r="B38" s="29" t="s">
+        <v>39</v>
+      </c>
+      <c r="C38" s="29" t="s">
+        <v>66</v>
+      </c>
+      <c r="D38" s="29" t="s">
+        <v>132</v>
+      </c>
+      <c r="E38" s="29" t="s">
+        <v>122</v>
+      </c>
+      <c r="F38" s="30" t="s">
+        <v>123</v>
+      </c>
+      <c r="G38" s="24"/>
+    </row>
+    <row r="39" customFormat="false" ht="70.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="24"/>
+      <c r="B39" s="24"/>
+      <c r="C39" s="24"/>
+      <c r="D39" s="24" t="s">
+        <v>133</v>
+      </c>
+      <c r="E39" s="21" t="s">
+        <v>130</v>
+      </c>
+      <c r="F39" s="23" t="s">
+        <v>86</v>
+      </c>
+      <c r="G39" s="24"/>
+    </row>
+    <row r="40" customFormat="false" ht="59" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="24"/>
+      <c r="B40" s="24"/>
+      <c r="C40" s="24"/>
+      <c r="D40" s="24" t="s">
+        <v>134</v>
+      </c>
+      <c r="E40" s="21" t="s">
         <v>74</v>
       </c>
-      <c r="G25" s="22"/>
-    </row>
-    <row r="26" customFormat="false" ht="24.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="27" t="s">
-        <v>30</v>
-      </c>
-      <c r="B26" s="27" t="s">
-        <v>31</v>
-      </c>
-      <c r="C26" s="27" t="s">
-        <v>65</v>
-      </c>
-      <c r="D26" s="27" t="s">
-        <v>106</v>
-      </c>
-      <c r="E26" s="27" t="s">
-        <v>107</v>
-      </c>
-      <c r="F26" s="28" t="s">
-        <v>108</v>
-      </c>
-      <c r="G26" s="22"/>
-    </row>
-    <row r="27" customFormat="false" ht="24.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="22"/>
-      <c r="B27" s="22"/>
-      <c r="C27" s="22"/>
-      <c r="D27" s="22" t="s">
-        <v>109</v>
-      </c>
-      <c r="E27" s="19" t="s">
-        <v>70</v>
-      </c>
-      <c r="F27" s="21" t="s">
-        <v>85</v>
-      </c>
-      <c r="G27" s="22"/>
-    </row>
-    <row r="28" customFormat="false" ht="47.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="22"/>
-      <c r="B28" s="22"/>
-      <c r="C28" s="22"/>
-      <c r="D28" s="22" t="s">
-        <v>110</v>
-      </c>
-      <c r="E28" s="19" t="s">
-        <v>73</v>
-      </c>
-      <c r="F28" s="21" t="s">
-        <v>111</v>
-      </c>
-      <c r="G28" s="22"/>
-    </row>
-    <row r="29" customFormat="false" ht="24.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="27" t="s">
-        <v>32</v>
-      </c>
-      <c r="B29" s="27" t="s">
-        <v>33</v>
-      </c>
-      <c r="C29" s="27" t="s">
-        <v>65</v>
-      </c>
-      <c r="D29" s="27" t="s">
-        <v>112</v>
-      </c>
-      <c r="E29" s="27" t="s">
-        <v>113</v>
-      </c>
-      <c r="F29" s="28" t="s">
-        <v>68</v>
-      </c>
-      <c r="G29" s="22"/>
-    </row>
-    <row r="30" customFormat="false" ht="12.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="22"/>
-      <c r="B30" s="22"/>
-      <c r="C30" s="22"/>
-      <c r="D30" s="22" t="s">
-        <v>114</v>
-      </c>
-      <c r="E30" s="19" t="s">
-        <v>115</v>
-      </c>
-      <c r="F30" s="21" t="s">
-        <v>116</v>
-      </c>
-      <c r="G30" s="22"/>
-    </row>
-    <row r="31" customFormat="false" ht="47.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="22"/>
-      <c r="B31" s="22"/>
-      <c r="C31" s="22"/>
-      <c r="D31" s="22" t="s">
-        <v>117</v>
-      </c>
-      <c r="E31" s="19" t="s">
-        <v>73</v>
-      </c>
-      <c r="F31" s="21" t="s">
-        <v>118</v>
-      </c>
-      <c r="G31" s="22"/>
-    </row>
-    <row r="32" customFormat="false" ht="87.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="27" t="s">
-        <v>34</v>
-      </c>
-      <c r="B32" s="27" t="s">
-        <v>35</v>
-      </c>
-      <c r="C32" s="27" t="s">
-        <v>65</v>
-      </c>
-      <c r="D32" s="27" t="s">
-        <v>119</v>
-      </c>
-      <c r="E32" s="27" t="s">
-        <v>120</v>
-      </c>
-      <c r="F32" s="28" t="s">
-        <v>121</v>
-      </c>
-      <c r="G32" s="22"/>
-    </row>
-    <row r="33" customFormat="false" ht="24.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="22"/>
-      <c r="B33" s="22"/>
-      <c r="C33" s="22"/>
-      <c r="D33" s="22" t="s">
-        <v>122</v>
-      </c>
-      <c r="E33" s="19" t="s">
-        <v>70</v>
-      </c>
-      <c r="F33" s="21" t="s">
-        <v>85</v>
-      </c>
-      <c r="G33" s="22"/>
-    </row>
-    <row r="34" customFormat="false" ht="59" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="22"/>
-      <c r="B34" s="22"/>
-      <c r="C34" s="22"/>
-      <c r="D34" s="22" t="s">
-        <v>123</v>
-      </c>
-      <c r="E34" s="19" t="s">
-        <v>73</v>
-      </c>
-      <c r="F34" s="21" t="s">
-        <v>124</v>
-      </c>
-      <c r="G34" s="22"/>
-    </row>
-    <row r="35" customFormat="false" ht="35.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="27" t="s">
-        <v>36</v>
-      </c>
-      <c r="B35" s="27" t="s">
-        <v>37</v>
-      </c>
-      <c r="C35" s="27" t="s">
-        <v>65</v>
-      </c>
-      <c r="D35" s="27" t="s">
-        <v>125</v>
-      </c>
-      <c r="E35" s="27" t="s">
-        <v>113</v>
-      </c>
-      <c r="F35" s="28" t="s">
+      <c r="F40" s="23" t="s">
         <v>126</v>
       </c>
-      <c r="G35" s="22"/>
-    </row>
-    <row r="36" customFormat="false" ht="71.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="22"/>
-      <c r="B36" s="22"/>
-      <c r="C36" s="22"/>
-      <c r="D36" s="22" t="s">
-        <v>127</v>
-      </c>
-      <c r="E36" s="19" t="s">
-        <v>128</v>
-      </c>
-      <c r="F36" s="21" t="s">
-        <v>85</v>
-      </c>
-      <c r="G36" s="22"/>
-    </row>
-    <row r="37" customFormat="false" ht="59" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="22"/>
-      <c r="B37" s="22"/>
-      <c r="C37" s="22"/>
-      <c r="D37" s="22" t="s">
-        <v>129</v>
-      </c>
-      <c r="E37" s="19" t="s">
-        <v>73</v>
-      </c>
-      <c r="F37" s="21" t="s">
-        <v>124</v>
-      </c>
-      <c r="G37" s="22"/>
-    </row>
-    <row r="38" customFormat="false" ht="87.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="27" t="s">
-        <v>38</v>
-      </c>
-      <c r="B38" s="27" t="s">
-        <v>39</v>
-      </c>
-      <c r="C38" s="27" t="s">
-        <v>65</v>
-      </c>
-      <c r="D38" s="27" t="s">
-        <v>130</v>
-      </c>
-      <c r="E38" s="27" t="s">
-        <v>120</v>
-      </c>
-      <c r="F38" s="28" t="s">
-        <v>121</v>
-      </c>
-      <c r="G38" s="22"/>
-    </row>
-    <row r="39" customFormat="false" ht="70.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="22"/>
-      <c r="B39" s="22"/>
-      <c r="C39" s="22"/>
-      <c r="D39" s="22" t="s">
-        <v>131</v>
-      </c>
-      <c r="E39" s="19" t="s">
-        <v>128</v>
-      </c>
-      <c r="F39" s="21" t="s">
-        <v>85</v>
-      </c>
-      <c r="G39" s="22"/>
-    </row>
-    <row r="40" customFormat="false" ht="59" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="22"/>
-      <c r="B40" s="22"/>
-      <c r="C40" s="22"/>
-      <c r="D40" s="22" t="s">
-        <v>132</v>
-      </c>
-      <c r="E40" s="19" t="s">
-        <v>73</v>
-      </c>
-      <c r="F40" s="21" t="s">
-        <v>124</v>
-      </c>
-      <c r="G40" s="22"/>
-    </row>
-    <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="27"/>
-      <c r="B41" s="27"/>
-      <c r="C41" s="27"/>
-      <c r="D41" s="27"/>
-      <c r="E41" s="27"/>
-      <c r="F41" s="27"/>
-      <c r="G41" s="22"/>
-    </row>
-    <row r="42" customFormat="false" ht="16.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="22"/>
-      <c r="B42" s="22"/>
-      <c r="C42" s="22"/>
-      <c r="D42" s="22"/>
-      <c r="E42" s="22"/>
-      <c r="F42" s="22"/>
-      <c r="G42" s="22"/>
-    </row>
-    <row r="43" customFormat="false" ht="16.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="30"/>
-      <c r="B43" s="30"/>
-      <c r="C43" s="30"/>
-      <c r="D43" s="30"/>
-      <c r="E43" s="30"/>
-      <c r="F43" s="30"/>
+      <c r="G40" s="24"/>
+    </row>
+    <row r="41" customFormat="false" ht="59" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="29" t="s">
+        <v>40</v>
+      </c>
+      <c r="B41" s="29" t="s">
+        <v>41</v>
+      </c>
+      <c r="C41" s="29" t="s">
+        <v>66</v>
+      </c>
+      <c r="D41" s="29" t="s">
+        <v>135</v>
+      </c>
+      <c r="E41" s="29" t="s">
+        <v>136</v>
+      </c>
+      <c r="F41" s="30" t="s">
+        <v>137</v>
+      </c>
+      <c r="G41" s="24"/>
+    </row>
+    <row r="42" customFormat="false" ht="70.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="24"/>
+      <c r="B42" s="24"/>
+      <c r="C42" s="24"/>
+      <c r="D42" s="24" t="s">
+        <v>138</v>
+      </c>
+      <c r="E42" s="21" t="s">
+        <v>139</v>
+      </c>
+      <c r="F42" s="23" t="s">
+        <v>140</v>
+      </c>
+      <c r="G42" s="24"/>
+    </row>
+    <row r="43" customFormat="false" ht="24.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="32"/>
+      <c r="B43" s="32"/>
+      <c r="C43" s="32"/>
+      <c r="D43" s="32" t="s">
+        <v>141</v>
+      </c>
+      <c r="E43" s="33" t="s">
+        <v>142</v>
+      </c>
+      <c r="F43" s="34" t="s">
+        <v>143</v>
+      </c>
     </row>
     <row r="44" customFormat="false" ht="16.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="30"/>
-      <c r="B44" s="30"/>
-      <c r="C44" s="30"/>
-      <c r="D44" s="30"/>
-      <c r="E44" s="30"/>
-      <c r="F44" s="30"/>
+      <c r="A44" s="35"/>
+      <c r="B44" s="35"/>
+      <c r="C44" s="35"/>
+      <c r="D44" s="35"/>
+      <c r="E44" s="35"/>
+      <c r="F44" s="35"/>
     </row>
     <row r="45" customFormat="false" ht="16.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="30"/>
-      <c r="B45" s="30"/>
-      <c r="C45" s="30"/>
-      <c r="D45" s="30"/>
-      <c r="E45" s="30"/>
-      <c r="F45" s="30"/>
+      <c r="A45" s="35"/>
+      <c r="B45" s="35"/>
+      <c r="C45" s="35"/>
+      <c r="D45" s="35"/>
+      <c r="E45" s="35"/>
+      <c r="F45" s="35"/>
     </row>
     <row r="46" customFormat="false" ht="16.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="30"/>
-      <c r="B46" s="30"/>
-      <c r="C46" s="30"/>
-      <c r="D46" s="30"/>
-      <c r="E46" s="30"/>
-      <c r="F46" s="30"/>
+      <c r="A46" s="35"/>
+      <c r="B46" s="35"/>
+      <c r="C46" s="35"/>
+      <c r="D46" s="35"/>
+      <c r="E46" s="35"/>
+      <c r="F46" s="35"/>
     </row>
     <row r="47" customFormat="false" ht="16.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="30"/>
-      <c r="B47" s="30"/>
-      <c r="C47" s="30"/>
-      <c r="D47" s="30"/>
-      <c r="E47" s="30"/>
-      <c r="F47" s="30"/>
+      <c r="A47" s="35"/>
+      <c r="B47" s="35"/>
+      <c r="C47" s="35"/>
+      <c r="D47" s="35"/>
+      <c r="E47" s="35"/>
+      <c r="F47" s="35"/>
     </row>
     <row r="48" customFormat="false" ht="16.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="30"/>
-      <c r="B48" s="30"/>
-      <c r="C48" s="30"/>
-      <c r="D48" s="30"/>
-      <c r="E48" s="30"/>
-      <c r="F48" s="30"/>
+      <c r="A48" s="35"/>
+      <c r="B48" s="35"/>
+      <c r="C48" s="35"/>
+      <c r="D48" s="35"/>
+      <c r="E48" s="35"/>
+      <c r="F48" s="35"/>
     </row>
     <row r="49" customFormat="false" ht="16.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="30"/>
-      <c r="B49" s="30"/>
-      <c r="C49" s="30"/>
-      <c r="D49" s="30"/>
-      <c r="E49" s="30"/>
-      <c r="F49" s="30"/>
+      <c r="A49" s="35"/>
+      <c r="B49" s="35"/>
+      <c r="C49" s="35"/>
+      <c r="D49" s="35"/>
+      <c r="E49" s="35"/>
+      <c r="F49" s="35"/>
     </row>
     <row r="50" customFormat="false" ht="16.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="30"/>
-      <c r="B50" s="30"/>
-      <c r="C50" s="30"/>
-      <c r="D50" s="30"/>
-      <c r="E50" s="30"/>
-      <c r="F50" s="30"/>
+      <c r="A50" s="35"/>
+      <c r="B50" s="35"/>
+      <c r="C50" s="35"/>
+      <c r="D50" s="35"/>
+      <c r="E50" s="35"/>
+      <c r="F50" s="35"/>
     </row>
     <row r="51" customFormat="false" ht="16.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="30"/>
-      <c r="B51" s="30"/>
-      <c r="C51" s="30"/>
-      <c r="D51" s="30"/>
-      <c r="E51" s="30"/>
-      <c r="F51" s="30"/>
+      <c r="A51" s="35"/>
+      <c r="B51" s="35"/>
+      <c r="C51" s="35"/>
+      <c r="D51" s="35"/>
+      <c r="E51" s="35"/>
+      <c r="F51" s="35"/>
     </row>
     <row r="52" customFormat="false" ht="16.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="30"/>
-      <c r="B52" s="30"/>
-      <c r="C52" s="30"/>
-      <c r="D52" s="30"/>
-      <c r="E52" s="30"/>
-      <c r="F52" s="30"/>
+      <c r="A52" s="35"/>
+      <c r="B52" s="35"/>
+      <c r="C52" s="35"/>
+      <c r="D52" s="35"/>
+      <c r="E52" s="35"/>
+      <c r="F52" s="35"/>
     </row>
     <row r="53" customFormat="false" ht="16.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="30"/>
-      <c r="B53" s="30"/>
-      <c r="C53" s="30"/>
-      <c r="D53" s="30"/>
-      <c r="E53" s="30"/>
-      <c r="F53" s="30"/>
+      <c r="A53" s="35"/>
+      <c r="B53" s="35"/>
+      <c r="C53" s="35"/>
+      <c r="D53" s="35"/>
+      <c r="E53" s="35"/>
+      <c r="F53" s="35"/>
     </row>
     <row r="54" customFormat="false" ht="16.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="30"/>
-      <c r="B54" s="30"/>
-      <c r="C54" s="30"/>
-      <c r="D54" s="30"/>
-      <c r="E54" s="30"/>
-      <c r="F54" s="30"/>
+      <c r="A54" s="35"/>
+      <c r="B54" s="35"/>
+      <c r="C54" s="35"/>
+      <c r="D54" s="35"/>
+      <c r="E54" s="35"/>
+      <c r="F54" s="35"/>
     </row>
     <row r="55" customFormat="false" ht="16.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="30"/>
-      <c r="B55" s="30"/>
-      <c r="C55" s="30"/>
-      <c r="D55" s="30"/>
-      <c r="E55" s="30"/>
-      <c r="F55" s="30"/>
+      <c r="A55" s="35"/>
+      <c r="B55" s="35"/>
+      <c r="C55" s="35"/>
+      <c r="D55" s="35"/>
+      <c r="E55" s="35"/>
+      <c r="F55" s="35"/>
     </row>
     <row r="56" customFormat="false" ht="16.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="30"/>
-      <c r="B56" s="30"/>
-      <c r="C56" s="30"/>
-      <c r="D56" s="30"/>
-      <c r="E56" s="30"/>
-      <c r="F56" s="30"/>
+      <c r="A56" s="35"/>
+      <c r="B56" s="35"/>
+      <c r="C56" s="35"/>
+      <c r="D56" s="35"/>
+      <c r="E56" s="35"/>
+      <c r="F56" s="35"/>
     </row>
     <row r="57" customFormat="false" ht="16.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="30"/>
-      <c r="B57" s="30"/>
-      <c r="C57" s="30"/>
-      <c r="D57" s="30"/>
-      <c r="E57" s="30"/>
-      <c r="F57" s="30"/>
+      <c r="A57" s="35"/>
+      <c r="B57" s="35"/>
+      <c r="C57" s="35"/>
+      <c r="D57" s="35"/>
+      <c r="E57" s="35"/>
+      <c r="F57" s="35"/>
     </row>
     <row r="58" customFormat="false" ht="16.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="30"/>
-      <c r="B58" s="30"/>
-      <c r="C58" s="30"/>
-      <c r="D58" s="30"/>
-      <c r="E58" s="30"/>
-      <c r="F58" s="30"/>
+      <c r="A58" s="35"/>
+      <c r="B58" s="35"/>
+      <c r="C58" s="35"/>
+      <c r="D58" s="35"/>
+      <c r="E58" s="35"/>
+      <c r="F58" s="35"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>